<commit_message>
n8n board refresh 2026-06-25T17:38:55Z
</commit_message>
<xml_diff>
--- a/app/reports/INTR_research.xlsx
+++ b/app/reports/INTR_research.xlsx
@@ -620,7 +620,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generated 2026-06-23 17:36 · Source: FMP · Methodology: financial-analysis plugin (Anthropic FSI), adapted for free-tier data</t>
+          <t>Generated 2026-06-25 17:36 · Source: FMP · Methodology: financial-analysis plugin (Anthropic FSI), adapted for free-tier data</t>
         </is>
       </c>
     </row>
@@ -689,7 +689,7 @@
         </is>
       </c>
       <c r="B9" s="7" t="n">
-        <v>5.26</v>
+        <v>5.305</v>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
@@ -879,7 +879,7 @@
         </is>
       </c>
       <c r="B5" s="9" t="n">
-        <v>0.04484999656677246</v>
+        <v>0.04383999824523926</v>
       </c>
     </row>
     <row r="6">
@@ -1208,7 +1208,7 @@
         </is>
       </c>
       <c r="B35" s="20" t="n">
-        <v>441488401.5209126</v>
+        <v>441488383.0348728</v>
       </c>
     </row>
     <row r="36">
@@ -1229,7 +1229,7 @@
         </is>
       </c>
       <c r="B37" s="22" t="n">
-        <v>5.26</v>
+        <v>5.305</v>
       </c>
     </row>
     <row r="38">
@@ -1508,14 +1508,14 @@
         </is>
       </c>
       <c r="C5" s="30" t="n">
-        <v>2322228992</v>
+        <v>2342095872</v>
       </c>
       <c r="D5" s="31" t="n">
-        <v>8.48</v>
+        <v>8.56</v>
       </c>
       <c r="E5" s="31" t="n"/>
       <c r="F5" s="31" t="n">
-        <v>2.45</v>
+        <v>2.44</v>
       </c>
     </row>
     <row r="6">
@@ -1530,14 +1530,14 @@
         </is>
       </c>
       <c r="C6" s="32" t="n">
-        <v>5614613504</v>
+        <v>5794084864</v>
       </c>
       <c r="D6" s="33" t="n">
-        <v>10.319444</v>
+        <v>10.649305</v>
       </c>
       <c r="E6" s="33" t="n"/>
       <c r="F6" s="33" t="n">
-        <v>5.454</v>
+        <v>5.571</v>
       </c>
     </row>
     <row r="7">
@@ -1552,14 +1552,14 @@
         </is>
       </c>
       <c r="C7" s="32" t="n">
-        <v>5121892864</v>
+        <v>5384415232</v>
       </c>
       <c r="D7" s="33" t="n">
-        <v>10.9671135</v>
+        <v>11.529232</v>
       </c>
       <c r="E7" s="33" t="n"/>
       <c r="F7" s="33" t="n">
-        <v>5.187</v>
+        <v>5.438</v>
       </c>
     </row>
     <row r="8">
@@ -1574,14 +1574,14 @@
         </is>
       </c>
       <c r="C8" s="32" t="n">
-        <v>3751935488</v>
+        <v>3824482048</v>
       </c>
       <c r="D8" s="33" t="n">
-        <v>15.302739</v>
+        <v>15.59863</v>
       </c>
       <c r="E8" s="33" t="n"/>
       <c r="F8" s="33" t="n">
-        <v>-1.21</v>
+        <v>-1.071</v>
       </c>
     </row>
     <row r="9">
@@ -1612,14 +1612,14 @@
         </is>
       </c>
       <c r="C10" s="32" t="n">
-        <v>4785616896</v>
+        <v>4984778752</v>
       </c>
       <c r="D10" s="33" t="n">
-        <v>18.152174</v>
+        <v>18.907608</v>
       </c>
       <c r="E10" s="33" t="n"/>
       <c r="F10" s="33" t="n">
-        <v>7.177</v>
+        <v>7.394</v>
       </c>
     </row>
     <row r="11">
@@ -1634,14 +1634,14 @@
         </is>
       </c>
       <c r="C11" s="32" t="n">
-        <v>4721421824</v>
+        <v>4793551872</v>
       </c>
       <c r="D11" s="33" t="n">
-        <v>11.332836</v>
+        <v>11.50597</v>
       </c>
       <c r="E11" s="33" t="n"/>
       <c r="F11" s="33" t="n">
-        <v>5.741</v>
+        <v>5.841</v>
       </c>
     </row>
     <row r="12">
@@ -1656,14 +1656,14 @@
         </is>
       </c>
       <c r="C12" s="32" t="n">
-        <v>33715314688</v>
+        <v>34511241216</v>
       </c>
       <c r="D12" s="33" t="n">
-        <v>12.926727</v>
+        <v>13.224467</v>
       </c>
       <c r="E12" s="33" t="n"/>
       <c r="F12" s="33" t="n">
-        <v>4.144</v>
+        <v>4.231</v>
       </c>
     </row>
     <row r="13">
@@ -1678,14 +1678,14 @@
         </is>
       </c>
       <c r="C13" s="32" t="n">
-        <v>4523895296</v>
+        <v>4711389184</v>
       </c>
       <c r="D13" s="33" t="n">
-        <v>13.97973</v>
+        <v>14.060359</v>
       </c>
       <c r="E13" s="33" t="n"/>
       <c r="F13" s="33" t="n">
-        <v>9.941000000000001</v>
+        <v>10.227</v>
       </c>
     </row>
     <row r="15">

</xml_diff>